<commit_message>
Test plan: clarify cart basics and single-item Buy now vs guest cart checkout
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Smart_Market_Test_Scenarios.xlsx
+++ b/docs/Smart_Market_Test_Scenarios.xlsx
@@ -1304,7 +1304,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -1360,8 +1359,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11" ht="26.25" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -1754,7 +1751,6 @@
         <v/>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
@@ -3836,7 +3832,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Header badge counts items; totals update; cart persists after reload; empty state when everything is removed.</t>
+          <t>Header badge counts items; totals update; cart persists after reload; the summary shows one orange "Checkout N items" button (whole cart) while each line keeps its own "Buy now"; empty state when everything is removed.</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
@@ -3866,7 +3862,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Checkout while logged out</t>
+          <t>Buy now (single item) while logged out</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -3887,7 +3883,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Login page, then back to the checkout of the same product.</t>
+          <t>Login page, then back to the checkout of the same product. Note: only the single-item "Buy now" needs an account; the whole-cart /checkout accepts guests (see CHK-13).</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Buy now accepts guests through the shared checkout
The single-item "Buy now" (/checkout/[slug]?qty=) now renders the same
checkout as the cart, so guests can order one listing with name + phone
and members keep the one-reference flow; the cart is left untouched.
Legacy ?order=<id> links still resume payment of pre-cart orders and stay
members-only. "Pay now" on grouped orders goes to the group page.

Also submits the guest phone shown as default in the delivery and Mobile
Money fields, and refreshes CHK-01/CHK-02 in the test plan.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Smart_Market_Test_Scenarios.xlsx
+++ b/docs/Smart_Market_Test_Scenarios.xlsx
@@ -3832,7 +3832,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Header badge counts items; totals update; cart persists after reload; the summary shows one orange "Checkout N items" button (whole cart) while each line keeps its own "Buy now"; empty state when everything is removed.</t>
+          <t>Header badge counts items; totals update; cart persists after reload; the summary shows one orange "Checkout N items" button (whole cart) while each line keeps its own "Buy now" (single item, same guest-capable checkout); empty state when everything is removed.</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
@@ -3862,18 +3862,22 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Buy now (single item) while logged out</t>
+          <t>Buy now while logged out (guest)</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Logged out, item in cart</t>
+          <t>Logged out</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
           <t>1.
-Click Buy now.</t>
+Open a product page and click Buy now.
+2.
+Fill the guest details (name, phone, optional email).
+3.
+Choose Cash on delivery, fill address and phone, place the order.</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -3883,7 +3887,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Login page, then back to the checkout of the same product. Note: only the single-item "Buy now" needs an account; the whole-cart /checkout accepts guests (see CHK-13).</t>
+          <t>The checkout opens directly with the "Your details" guest form (no login page); the order is confirmed with an SM-XXXXXX reference and a tracking link; "Have an account? Sign in" returns to the same checkout after login. Older "Pay now" links with ?order= still require an account.</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
@@ -3893,7 +3897,7 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J39" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Test plan: point staging URLs at smartplaze.com
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Smart_Market_Test_Scenarios.xlsx
+++ b/docs/Smart_Market_Test_Scenarios.xlsx
@@ -1300,10 +1300,11 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Staging: https://smartmarket.31.97.53.16.nip.io   ·   Generated 2026-09-24   ·   Fill the blue cells on the Scenarios sheet (Status, Actual result, Tester / date).</t>
-        </is>
-      </c>
-    </row>
+          <t>Staging: https://smartplaze.com   ·   Generated 2026-09-24   ·   Fill the blue cells on the Scenarios sheet (Status, Actual result, Tester / date).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -1359,6 +1360,8 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="26.25" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -1751,6 +1754,7 @@
         <v/>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
@@ -7498,7 +7502,7 @@
       <c r="E108" s="3" t="inlineStr">
         <is>
           <t>1.
-Open http://smartmarket.31.97.53.16.nip.io.</t>
+Open http://smartplaze.com.</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
@@ -8218,6 +8222,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -8372,6 +8377,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="16.85" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
@@ -8387,7 +8393,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://smartmarket.31.97.53.16.nip.io  (French: /fr)</t>
+          <t>https://smartplaze.com  (French: /fr)</t>
         </is>
       </c>
       <c r="C12" s="5" t="n"/>
@@ -8401,7 +8407,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://smartmarket.31.97.53.16.nip.io/admin</t>
+          <t>https://smartplaze.com/admin</t>
         </is>
       </c>
       <c r="C13" s="5" t="n"/>
@@ -8415,7 +8421,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://smartmarket.31.97.53.16.nip.io/seller</t>
+          <t>https://smartplaze.com/seller</t>
         </is>
       </c>
       <c r="C14" s="5" t="n"/>
@@ -8457,7 +8463,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Add https://smartmarket.31.97.53.16.nip.io/api/auth/google/callback as an authorised redirect URI in Google Cloud Console before testing.</t>
+          <t>Add https://api.smartplaze.com/api/auth/google/callback as an authorised redirect URI in Google Cloud Console before testing.</t>
         </is>
       </c>
       <c r="C17" s="5" t="n"/>

</xml_diff>